<commit_message>
design: integrar almacenamiento aprobado y calculos justificados
</commit_message>
<xml_diff>
--- a/calculos/calculos_y_restricciones.xlsx
+++ b/calculos/calculos_y_restricciones.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="R6df79bba42eb419b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="R347e8417d3d643f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="R949006f1efdb4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="R928caf0751474268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="Rb236232de79e4305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rd7c633aaad2945d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,12 +44,22 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF18354A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -74,7 +84,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="21">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -110,10 +120,56 @@
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="2">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -331,7 +387,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Dimensionamiento de la cámara</x:v>
+        <x:v>Dimensionamiento de componentes</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -341,7 +397,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Referencia: MQ022HG-IM-SM5X5-7NIR2. RAW16 sin compresión. MB decimales.</x:v>
+        <x:v>Cámara, almacenamiento y computador. MB y GB decimales; supuestos en Entradas.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -663,15 +719,15 @@
       <x:c r="A26" s="2" t="str">
         <x:v>Capacidad útil mínima de misión</x:v>
       </x:c>
-      <x:c r="B26" s="10" t="str">
-        <x:f>IF(AND(ISNUMBER(B13),COUNT('Entradas'!B24:B26)=3),(B13*'Entradas'!B24)/1000000+'Entradas'!B25+'Entradas'!B26,"Pendiente")</x:f>
-        <x:v>Pendiente</x:v>
+      <x:c r="B26" s="10" t="n">
+        <x:f>B44*1000</x:f>
+        <x:v>12201.6064</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
         <x:v>MB</x:v>
       </x:c>
       <x:c r="D26" s="6" t="str">
-        <x:v>Datos previos + generación × días + reserva.</x:v>
+        <x:v>Véase almacenamiento: cuotas aprobadas, resultados y reservas.</x:v>
       </x:c>
       <x:c r="E26" s="2"/>
       <x:c r="F26" s="2"/>
@@ -806,7 +862,514 @@
       <x:c r="E37" s="2"/>
       <x:c r="F37" s="2"/>
     </x:row>
+    <x:row r="38" ht="34" customHeight="1">
+      <x:c r="A38" s="6" t="str">
+        <x:v>Almacenamiento de misión</x:v>
+      </x:c>
+      <x:c r="B38" s="6"/>
+      <x:c r="C38" s="6"/>
+      <x:c r="D38" s="6"/>
+    </x:row>
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="15" t="str">
+        <x:v>Resultado</x:v>
+      </x:c>
+      <x:c r="B39" s="15" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C39" s="15" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D39" s="15" t="str">
+        <x:v>Justificación / alcance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="6" t="str">
+        <x:v>Imágenes RAW diarias</x:v>
+      </x:c>
+      <x:c r="B40" s="16" t="n">
+        <x:f>B11</x:f>
+        <x:v>44.56448</x:v>
+      </x:c>
+      <x:c r="C40" s="6" t="str">
+        <x:v>MB/día</x:v>
+      </x:c>
+      <x:c r="D40" s="6" t="str">
+        <x:v>Escenario de cámara existente; no vídeo continuo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="6" t="str">
+        <x:v>Cuota de resultados</x:v>
+      </x:c>
+      <x:c r="B41" s="16" t="n">
+        <x:f>B40*'Entradas'!B46</x:f>
+        <x:v>44.56448</x:v>
+      </x:c>
+      <x:c r="C41" s="6" t="str">
+        <x:v>MB/día</x:v>
+      </x:c>
+      <x:c r="D41" s="6" t="str">
+        <x:v>Se conserva además del RAW; no redundancia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="6" t="str">
+        <x:v>Cuota de auxiliares</x:v>
+      </x:c>
+      <x:c r="B42" s="16" t="n">
+        <x:f>'Entradas'!B47</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C42" s="6" t="str">
+        <x:v>MB/día</x:v>
+      </x:c>
+      <x:c r="D42" s="6" t="str">
+        <x:v>Presupuesto conjunto; no medición de telemetría.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="34" customHeight="1">
+      <x:c r="A43" s="6" t="str">
+        <x:v>Generación presupuestada</x:v>
+      </x:c>
+      <x:c r="B43" s="16" t="n">
+        <x:f>SUM(B40:B42)</x:f>
+        <x:v>91.12896</x:v>
+      </x:c>
+      <x:c r="C43" s="6" t="str">
+        <x:v>MB/día</x:v>
+      </x:c>
+      <x:c r="D43" s="6" t="str">
+        <x:v>RAW + resultados + auxiliares.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="6" t="str">
+        <x:v>Capacidad útil requerida</x:v>
+      </x:c>
+      <x:c r="B44" s="16" t="n">
+        <x:f>'Entradas'!B26/1000+B43*'Entradas'!B24/1000+'Entradas'!B25/1000</x:f>
+        <x:v>12.201606400000001</x:v>
+      </x:c>
+      <x:c r="C44" s="6" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="D44" s="6" t="str">
+        <x:v>Ocupación inicial + generación × días + reserva.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="6" t="str">
+        <x:v>Margen adicional a la reserva</x:v>
+      </x:c>
+      <x:c r="B45" s="16" t="n">
+        <x:f>'Entradas'!B49-B44</x:f>
+        <x:v>2.798393599999999</x:v>
+      </x:c>
+      <x:c r="C45" s="6" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="D45" s="6" t="str">
+        <x:v>La reserva libre ya está incluida en B44.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="6" t="str">
+        <x:v>Comparación con umbral útil</x:v>
+      </x:c>
+      <x:c r="B46" s="16" t="str">
+        <x:f>IF(B45&gt;=0,"Cumple escenario","No cumple")</x:f>
+        <x:v>Cumple escenario</x:v>
+      </x:c>
+      <x:c r="C46" s="6" t="str">
+        <x:v>estado</x:v>
+      </x:c>
+      <x:c r="D46" s="6" t="str">
+        <x:v>Condicional a capacidad útil real y cuotas; no ensayo físico.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="6" t="str">
+        <x:v>Capacidad nominal</x:v>
+      </x:c>
+      <x:c r="B47" s="16" t="n">
+        <x:f>'Entradas'!B48</x:f>
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C47" s="6" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="D47" s="6" t="str">
+        <x:v>Fabricante; distinta del espacio útil tras formato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="6" t="str">
+        <x:v>Capacidad útil exigida</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="n">
+        <x:f>'Entradas'!B49</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C48" s="6" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="D48" s="6" t="str">
+        <x:v>Umbral de aceptación; no medición.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="6" t="str">
+        <x:v>Límite aritmético de retención</x:v>
+      </x:c>
+      <x:c r="B49" s="16" t="n">
+        <x:f>IF(B43&gt;0,('Entradas'!B49-('Entradas'!B26+'Entradas'!B25)/1000)*1000/B43,"Sin generación")</x:f>
+        <x:v>120.70806031364782</x:v>
+      </x:c>
+      <x:c r="C49" s="6" t="str">
+        <x:v>días</x:v>
+      </x:c>
+      <x:c r="D49" s="6" t="str">
+        <x:v>Con cuotas y ocupación inicial dadas; no retención física NAND.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="6" t="str">
+        <x:v>Escritura lógica anual</x:v>
+      </x:c>
+      <x:c r="B50" s="16" t="n">
+        <x:f>B43*'Entradas'!B55/1000</x:f>
+        <x:v>33.262070400000006</x:v>
+      </x:c>
+      <x:c r="C50" s="6" t="str">
+        <x:v>GB/año</x:v>
+      </x:c>
+      <x:c r="D50" s="6" t="str">
+        <x:v>No equivale a desgaste físico ni TBW garantizado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="34" customHeight="1">
+      <x:c r="A51" s="6" t="str">
+        <x:v>Techo bruto del bus SD</x:v>
+      </x:c>
+      <x:c r="B51" s="16" t="n">
+        <x:f>'Entradas'!B50*'Entradas'!B51/8</x:f>
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="C51" s="6" t="str">
+        <x:v>MB/s</x:v>
+      </x:c>
+      <x:c r="D51" s="6" t="str">
+        <x:v>No velocidad sostenida de archivo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="34" customHeight="1">
+      <x:c r="A52" s="6" t="str">
+        <x:v>Escritura útil objetivo</x:v>
+      </x:c>
+      <x:c r="B52" s="16" t="n">
+        <x:f>B8*(1+'Entradas'!B46)/'Entradas'!B52/1000000</x:f>
+        <x:v>4.456448</x:v>
+      </x:c>
+      <x:c r="C52" s="6" t="str">
+        <x:v>MB/s</x:v>
+      </x:c>
+      <x:c r="D52" s="6" t="str">
+        <x:v>RAW + resultado por adquisición en el tiempo objetivo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="34" customHeight="1">
+      <x:c r="A53" s="6" t="str">
+        <x:v>Potencia máxima de microSD</x:v>
+      </x:c>
+      <x:c r="B53" s="16" t="str">
+        <x:f>IF(ISNUMBER('Entradas'!B54),'Entradas'!B53*'Entradas'!B54,"Pendiente")</x:f>
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="C53" s="6" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D53" s="6" t="str">
+        <x:v>Falta corriente máxima y arranque; no asumir cero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="34" customHeight="1">
+      <x:c r="A54" s="6"/>
+      <x:c r="B54" s="6"/>
+      <x:c r="C54" s="6"/>
+      <x:c r="D54" s="6"/>
+    </x:row>
+    <x:row r="55" ht="30" customHeight="1">
+      <x:c r="A55" s="15" t="str">
+        <x:v>Retención (días)</x:v>
+      </x:c>
+      <x:c r="B55" s="15" t="str">
+        <x:v>Requerida (GB)</x:v>
+      </x:c>
+      <x:c r="C55" s="15" t="str">
+        <x:v>Margen (GB)</x:v>
+      </x:c>
+      <x:c r="D55" s="15" t="str">
+        <x:v>Comparación con umbral útil</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="34" customHeight="1">
+      <x:c r="A56" s="6" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B56" s="16" t="n">
+        <x:f>'Entradas'!$B$26/1000+$B$43*A56/1000+'Entradas'!$B$25/1000</x:f>
+        <x:v>6.7338688</x:v>
+      </x:c>
+      <x:c r="C56" s="16" t="n">
+        <x:f>'Entradas'!$B$49-B56</x:f>
+        <x:v>8.2661312</x:v>
+      </x:c>
+      <x:c r="D56" s="6" t="str">
+        <x:f>IF(C56&gt;=0,"Cumple escenario","No cumple")</x:f>
+        <x:v>Cumple escenario</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="34" customHeight="1">
+      <x:c r="A57" s="6" t="n">
+        <x:f>'Entradas'!B24</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B57" s="16" t="n">
+        <x:f>'Entradas'!$B$26/1000+$B$43*A57/1000+'Entradas'!$B$25/1000</x:f>
+        <x:v>12.201606400000001</x:v>
+      </x:c>
+      <x:c r="C57" s="16" t="n">
+        <x:f>'Entradas'!$B$49-B57</x:f>
+        <x:v>2.798393599999999</x:v>
+      </x:c>
+      <x:c r="D57" s="6" t="str">
+        <x:f>IF(C57&gt;=0,"Cumple escenario","No cumple")</x:f>
+        <x:v>Cumple escenario</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="34" customHeight="1">
+      <x:c r="A58" s="6" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="B58" s="16" t="n">
+        <x:f>'Entradas'!$B$26/1000+$B$43*A58/1000+'Entradas'!$B$25/1000</x:f>
+        <x:v>20.403212800000002</x:v>
+      </x:c>
+      <x:c r="C58" s="16" t="n">
+        <x:f>'Entradas'!$B$49-B58</x:f>
+        <x:v>-5.403212800000002</x:v>
+      </x:c>
+      <x:c r="D58" s="6" t="str">
+        <x:f>IF(C58&gt;=0,"Cumple escenario","No cumple")</x:f>
+        <x:v>No cumple</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="34" customHeight="1">
+      <x:c r="A59" s="6"/>
+      <x:c r="B59" s="6"/>
+      <x:c r="C59" s="6"/>
+      <x:c r="D59" s="6"/>
+    </x:row>
+    <x:row r="60" ht="34" customHeight="1">
+      <x:c r="A60" s="6"/>
+      <x:c r="B60" s="6"/>
+      <x:c r="C60" s="6"/>
+      <x:c r="D60" s="6"/>
+    </x:row>
+    <x:row r="61" ht="34" customHeight="1">
+      <x:c r="A61" s="6"/>
+      <x:c r="B61" s="6"/>
+      <x:c r="C61" s="6"/>
+      <x:c r="D61" s="6"/>
+    </x:row>
+    <x:row r="62" ht="34" customHeight="1">
+      <x:c r="A62" s="6" t="str">
+        <x:v>Computador: capacidad de alimentación y recursos</x:v>
+      </x:c>
+      <x:c r="B62" s="6"/>
+      <x:c r="C62" s="6"/>
+      <x:c r="D62" s="6"/>
+    </x:row>
+    <x:row r="63" ht="30" customHeight="1">
+      <x:c r="A63" s="15" t="str">
+        <x:v>Resultado</x:v>
+      </x:c>
+      <x:c r="B63" s="15" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C63" s="15" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D63" s="15" t="str">
+        <x:v>Justificación / alcance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="34" customHeight="1">
+      <x:c r="A64" s="6" t="str">
+        <x:v>Tensión mínima SoM</x:v>
+      </x:c>
+      <x:c r="B64" s="16" t="n">
+        <x:f>'Entradas'!B56*(1-'Entradas'!B57)</x:f>
+        <x:v>4.75</x:v>
+      </x:c>
+      <x:c r="C64" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D64" s="6" t="str">
+        <x:v>Tensión exigida en pines VCC.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="34" customHeight="1">
+      <x:c r="A65" s="6" t="str">
+        <x:v>Tensión máxima SoM</x:v>
+      </x:c>
+      <x:c r="B65" s="16" t="n">
+        <x:f>'Entradas'!B56*(1+'Entradas'!B57)</x:f>
+        <x:v>5.25</x:v>
+      </x:c>
+      <x:c r="C65" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D65" s="6" t="str">
+        <x:v>Dentro de 3,135–5,5 V recomendados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="34" customHeight="1">
+      <x:c r="A66" s="6" t="str">
+        <x:v>Corriente sostenida de diseño</x:v>
+      </x:c>
+      <x:c r="B66" s="16" t="n">
+        <x:f>'Entradas'!B58/B64</x:f>
+        <x:v>1.736842105263158</x:v>
+      </x:c>
+      <x:c r="C66" s="6" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D66" s="6" t="str">
+        <x:v>Envolvente de familia / tensión mínima.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="34" customHeight="1">
+      <x:c r="A67" s="6" t="str">
+        <x:v>Corriente de pico de diseño</x:v>
+      </x:c>
+      <x:c r="B67" s="16" t="n">
+        <x:f>'Entradas'!B59/B64</x:f>
+        <x:v>2.6315789473684212</x:v>
+      </x:c>
+      <x:c r="C67" s="6" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D67" s="6" t="str">
+        <x:v>No consumo observado de nuestra revisión.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="34" customHeight="1">
+      <x:c r="A68" s="6" t="str">
+        <x:v>Capacidad a tensión mínima</x:v>
+      </x:c>
+      <x:c r="B68" s="16" t="n">
+        <x:f>B64*'Entradas'!B60</x:f>
+        <x:v>14.25</x:v>
+      </x:c>
+      <x:c r="C68" s="6" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D68" s="6" t="str">
+        <x:v>Rama exclusiva de computador.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="34" customHeight="1">
+      <x:c r="A69" s="6" t="str">
+        <x:v>Margen sobre envolvente pico</x:v>
+      </x:c>
+      <x:c r="B69" s="17" t="n">
+        <x:f>B68/'Entradas'!B59-1</x:f>
+        <x:v>0.1399999999999999</x:v>
+      </x:c>
+      <x:c r="C69" s="6" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="D69" s="6" t="str">
+        <x:v>No asignar este margen a cargas externas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="34" customHeight="1">
+      <x:c r="A70" s="6" t="str">
+        <x:v>Buffers RAW</x:v>
+      </x:c>
+      <x:c r="B70" s="20" t="n">
+        <x:f>B8*'Entradas'!B64</x:f>
+        <x:v>8912896</x:v>
+      </x:c>
+      <x:c r="C70" s="6" t="str">
+        <x:v>bytes</x:v>
+      </x:c>
+      <x:c r="D70" s="6" t="str">
+        <x:v>No incluye Linux, SDK ni algoritmo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="34" customHeight="1">
+      <x:c r="A71" s="6" t="str">
+        <x:v>Área proyectada módulo</x:v>
+      </x:c>
+      <x:c r="B71" s="16" t="n">
+        <x:f>'Entradas'!B61*'Entradas'!B62</x:f>
+        <x:v>2436</x:v>
+      </x:c>
+      <x:c r="C71" s="6" t="str">
+        <x:v>mm²</x:v>
+      </x:c>
+      <x:c r="D71" s="6" t="str">
+        <x:v>Solo proyección del módulo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="34" customHeight="1">
+      <x:c r="A72" s="6" t="str">
+        <x:v>Fracción de área de PCB</x:v>
+      </x:c>
+      <x:c r="B72" s="17" t="n">
+        <x:f>B71/('Entradas'!B63^2)</x:f>
+        <x:v>0.30074074074074075</x:v>
+      </x:c>
+      <x:c r="C72" s="6" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="D72" s="6" t="str">
+        <x:v>No demuestra encaje con RF y disipación.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="34" customHeight="1">
+      <x:c r="A73" s="6"/>
+      <x:c r="B73" s="6"/>
+      <x:c r="C73" s="6"/>
+      <x:c r="D73" s="6"/>
+    </x:row>
+    <x:row r="74" ht="34" customHeight="1">
+      <x:c r="A74" s="6"/>
+      <x:c r="B74" s="6"/>
+      <x:c r="C74" s="6"/>
+      <x:c r="D74" s="6"/>
+    </x:row>
+    <x:row r="75" ht="34" customHeight="1">
+      <x:c r="A75" s="6"/>
+      <x:c r="B75" s="6"/>
+      <x:c r="C75" s="6"/>
+      <x:c r="D75" s="6"/>
+    </x:row>
   </x:sheetData>
+  <x:conditionalFormatting sqref="B45:B45">
+    <x:cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <x:formula>0</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C56:C58">
+    <x:cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <x:formula>0</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -836,7 +1399,7 @@
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Cámara XIMEA: datos y supuestos</x:v>
+        <x:v>Datos y supuestos de componentes</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -846,7 +1409,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>Selección eléctrica académica. Consulta: 2026-10-24. Amarillo: supuestos o datos por completar.</x:v>
+        <x:v>Actualización: 2026-10-25. Amarillo: decisiones editables o datos por completar.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1240,54 +1803,60 @@
       <x:c r="A24" s="6" t="str">
         <x:v>Retención sin descarga</x:v>
       </x:c>
-      <x:c r="B24" s="8"/>
+      <x:c r="B24" s="8" t="n">
+        <x:v>90</x:v>
+      </x:c>
       <x:c r="C24" s="6" t="str">
         <x:v>días</x:v>
       </x:c>
       <x:c r="D24" s="6" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Supuesto aprobado</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
-        <x:v>Misión futura</x:v>
+        <x:v>Acuerdo 2026-10-25</x:v>
       </x:c>
       <x:c r="F24" s="6" t="str">
-        <x:v>Falta acordar autonomía requerida</x:v>
+        <x:v>Contingencia sin descarga; no resultado orbital</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="43" customHeight="1">
       <x:c r="A25" s="6" t="str">
         <x:v>Reserva de almacenamiento</x:v>
       </x:c>
-      <x:c r="B25" s="8"/>
+      <x:c r="B25" s="8" t="n">
+        <x:v>3000</x:v>
+      </x:c>
       <x:c r="C25" s="6" t="str">
         <x:v>MB</x:v>
       </x:c>
       <x:c r="D25" s="6" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Reserva aprobada</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
-        <x:v>Por dimensionar</x:v>
+        <x:v>Acuerdo 2026-10-25</x:v>
       </x:c>
       <x:c r="F25" s="6" t="str">
-        <x:v>Reserva adicional libre</x:v>
+        <x:v>Debe permanecer libre; no volver a sumar</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="43" customHeight="1">
       <x:c r="A26" s="6" t="str">
         <x:v>Datos previos almacenados</x:v>
       </x:c>
-      <x:c r="B26" s="8"/>
+      <x:c r="B26" s="8" t="n">
+        <x:v>1000</x:v>
+      </x:c>
       <x:c r="C26" s="6" t="str">
         <x:v>MB</x:v>
       </x:c>
       <x:c r="D26" s="6" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Límite aprobado</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
-        <x:v>Escenario futuro</x:v>
+        <x:v>Acuerdo 2026-10-25</x:v>
       </x:c>
       <x:c r="F26" s="6" t="str">
-        <x:v>Falta definir ocupación inicial</x:v>
+        <x:v>Máximo al comenzar la contingencia</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26" customHeight="1">
@@ -1451,6 +2020,562 @@
       <x:c r="D43" s="2"/>
       <x:c r="E43" s="2"/>
       <x:c r="F43" s="2"/>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="15" t="str">
+        <x:v>Parámetro</x:v>
+      </x:c>
+      <x:c r="B45" s="15" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C45" s="15" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D45" s="15" t="str">
+        <x:v>Tipo</x:v>
+      </x:c>
+      <x:c r="E45" s="15" t="str">
+        <x:v>Fuente</x:v>
+      </x:c>
+      <x:c r="F45" s="15" t="str">
+        <x:v>Justificación / alcance</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="50" customHeight="1">
+      <x:c r="A46" s="6" t="str">
+        <x:v>Cuota de resultados / RAW</x:v>
+      </x:c>
+      <x:c r="B46" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C46" s="6" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="D46" s="6" t="str">
+        <x:v>Supuesto aprobado</x:v>
+      </x:c>
+      <x:c r="E46" s="6" t="str">
+        <x:v>Acuerdo 2026-10-25</x:v>
+      </x:c>
+      <x:c r="F46" s="6" t="str">
+        <x:v>Espacio para derivados; no copia redundante ni algoritmo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="50" customHeight="1">
+      <x:c r="A47" s="6" t="str">
+        <x:v>Cuota de auxiliares diarios</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C47" s="6" t="str">
+        <x:v>MB/día</x:v>
+      </x:c>
+      <x:c r="D47" s="6" t="str">
+        <x:v>Supuesto aprobado</x:v>
+      </x:c>
+      <x:c r="E47" s="6" t="str">
+        <x:v>Acuerdo 2026-10-25</x:v>
+      </x:c>
+      <x:c r="F47" s="6" t="str">
+        <x:v>Metadatos, telemetría, índices y eventos; no medición</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="50" customHeight="1">
+      <x:c r="A48" s="6" t="str">
+        <x:v>Capacidad nominal microSD</x:v>
+      </x:c>
+      <x:c r="B48" s="16" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C48" s="6" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="D48" s="6" t="str">
+        <x:v>Fabricante</x:v>
+      </x:c>
+      <x:c r="E48" s="6" t="str">
+        <x:v>SRC-012</x:v>
+      </x:c>
+      <x:c r="F48" s="6" t="str">
+        <x:v>SDCIT2/16GBSP; no es capacidad útil</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="50" customHeight="1">
+      <x:c r="A49" s="6" t="str">
+        <x:v>Umbral de capacidad útil</x:v>
+      </x:c>
+      <x:c r="B49" s="18" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C49" s="6" t="str">
+        <x:v>GB</x:v>
+      </x:c>
+      <x:c r="D49" s="6" t="str">
+        <x:v>Criterio de aceptación</x:v>
+      </x:c>
+      <x:c r="E49" s="6" t="str">
+        <x:v>Acuerdo 2026-10-25</x:v>
+      </x:c>
+      <x:c r="F49" s="6" t="str">
+        <x:v>Comprobar tras formato; no capacidad medida</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="50" customHeight="1">
+      <x:c r="A50" s="6" t="str">
+        <x:v>Ancho de bus SD</x:v>
+      </x:c>
+      <x:c r="B50" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C50" s="6" t="str">
+        <x:v>bits</x:v>
+      </x:c>
+      <x:c r="D50" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E50" s="6" t="str">
+        <x:v>SRC-009 §5.14</x:v>
+      </x:c>
+      <x:c r="F50" s="6" t="str">
+        <x:v>USDHC2 externo; eMMC interna independiente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="50" customHeight="1">
+      <x:c r="A51" s="6" t="str">
+        <x:v>Reloj SD objetivo</x:v>
+      </x:c>
+      <x:c r="B51" s="18" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C51" s="6" t="str">
+        <x:v>MHz</x:v>
+      </x:c>
+      <x:c r="D51" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E51" s="6" t="str">
+        <x:v>SRC-009 tabla 52</x:v>
+      </x:c>
+      <x:c r="F51" s="6" t="str">
+        <x:v>Default Speed; señalización 3,3 V</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="50" customHeight="1">
+      <x:c r="A52" s="6" t="str">
+        <x:v>Tiempo objetivo RAW + resultado</x:v>
+      </x:c>
+      <x:c r="B52" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C52" s="6" t="str">
+        <x:v>s</x:v>
+      </x:c>
+      <x:c r="D52" s="6" t="str">
+        <x:v>Criterio de diseño</x:v>
+      </x:c>
+      <x:c r="E52" s="6" t="str">
+        <x:v>Acuerdo 2026-10-25</x:v>
+      </x:c>
+      <x:c r="F52" s="6" t="str">
+        <x:v>Objetivo a comprobar; no latencia garantizada</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="50" customHeight="1">
+      <x:c r="A53" s="6" t="str">
+        <x:v>Alimentación microSD</x:v>
+      </x:c>
+      <x:c r="B53" s="16" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="C53" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D53" s="6" t="str">
+        <x:v>Fabricante</x:v>
+      </x:c>
+      <x:c r="E53" s="6" t="str">
+        <x:v>SRC-012</x:v>
+      </x:c>
+      <x:c r="F53" s="6" t="str">
+        <x:v>Rama independiente de la reserva del SoM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="50" customHeight="1">
+      <x:c r="A54" s="6" t="str">
+        <x:v>Corriente máxima microSD</x:v>
+      </x:c>
+      <x:c r="B54" s="18"/>
+      <x:c r="C54" s="6" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D54" s="6" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="E54" s="6" t="str">
+        <x:v>SRC-012 no informa</x:v>
+      </x:c>
+      <x:c r="F54" s="6" t="str">
+        <x:v>No usar un valor típico o inventado como máximo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="50" customHeight="1">
+      <x:c r="A55" s="6" t="str">
+        <x:v>Período anual de cálculo</x:v>
+      </x:c>
+      <x:c r="B55" s="18" t="n">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="C55" s="6" t="str">
+        <x:v>días</x:v>
+      </x:c>
+      <x:c r="D55" s="6" t="str">
+        <x:v>Convención</x:v>
+      </x:c>
+      <x:c r="E55" s="6" t="str">
+        <x:v>Definición</x:v>
+      </x:c>
+      <x:c r="F55" s="6" t="str">
+        <x:v>Volumen lógico; no amplificación de NAND</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="50" customHeight="1">
+      <x:c r="A56" s="6" t="str">
+        <x:v>Tensión nominal del SoM</x:v>
+      </x:c>
+      <x:c r="B56" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C56" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D56" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E56" s="6" t="str">
+        <x:v>SEL-002</x:v>
+      </x:c>
+      <x:c r="F56" s="6" t="str">
+        <x:v>Garantizar tolerancia en VCC tras caídas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="50" customHeight="1">
+      <x:c r="A57" s="6" t="str">
+        <x:v>Tolerancia de tensión SoM</x:v>
+      </x:c>
+      <x:c r="B57" s="19" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C57" s="6" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="D57" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E57" s="6" t="str">
+        <x:v>SEL-002</x:v>
+      </x:c>
+      <x:c r="F57" s="6" t="str">
+        <x:v>Compatible con rango recomendado de SRC-009</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="50" customHeight="1">
+      <x:c r="A58" s="6" t="str">
+        <x:v>Envolvente sostenida Verdin</x:v>
+      </x:c>
+      <x:c r="B58" s="16" t="n">
+        <x:v>8.25</x:v>
+      </x:c>
+      <x:c r="C58" s="6" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D58" s="6" t="str">
+        <x:v>Guía de familia</x:v>
+      </x:c>
+      <x:c r="E58" s="6" t="str">
+        <x:v>SRC-011 §3.1</x:v>
+      </x:c>
+      <x:c r="F58" s="6" t="str">
+        <x:v>Dimensionamiento; no consumo de nuestra aplicación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="50" customHeight="1">
+      <x:c r="A59" s="6" t="str">
+        <x:v>Envolvente de pico Verdin</x:v>
+      </x:c>
+      <x:c r="B59" s="16" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="C59" s="6" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D59" s="6" t="str">
+        <x:v>Guía de familia</x:v>
+      </x:c>
+      <x:c r="E59" s="6" t="str">
+        <x:v>SRC-011 §3.1</x:v>
+      </x:c>
+      <x:c r="F59" s="6" t="str">
+        <x:v>Dimensionar fuente para esta envolvente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="50" customHeight="1">
+      <x:c r="A60" s="6" t="str">
+        <x:v>Capacidad de corriente rama SoM</x:v>
+      </x:c>
+      <x:c r="B60" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C60" s="6" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D60" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E60" s="6" t="str">
+        <x:v>SEL-002</x:v>
+      </x:c>
+      <x:c r="F60" s="6" t="str">
+        <x:v>Solo SoM; excluye cámara, radio y memoria externa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="50" customHeight="1">
+      <x:c r="A61" s="6" t="str">
+        <x:v>Largo proyectado SoM</x:v>
+      </x:c>
+      <x:c r="B61" s="16" t="n">
+        <x:v>69.6</x:v>
+      </x:c>
+      <x:c r="C61" s="6" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D61" s="6" t="str">
+        <x:v>Fabricante</x:v>
+      </x:c>
+      <x:c r="E61" s="6" t="str">
+        <x:v>SRC-009 §8.5</x:v>
+      </x:c>
+      <x:c r="F61" s="6" t="str">
+        <x:v>Excluye fijaciones y zócalo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="50" customHeight="1">
+      <x:c r="A62" s="6" t="str">
+        <x:v>Ancho proyectado SoM</x:v>
+      </x:c>
+      <x:c r="B62" s="16" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C62" s="6" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D62" s="6" t="str">
+        <x:v>Fabricante</x:v>
+      </x:c>
+      <x:c r="E62" s="6" t="str">
+        <x:v>SRC-009 §8.5</x:v>
+      </x:c>
+      <x:c r="F62" s="6" t="str">
+        <x:v>Excluye disipación y zonas libres</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="50" customHeight="1">
+      <x:c r="A63" s="6" t="str">
+        <x:v>Lado de PCB de referencia</x:v>
+      </x:c>
+      <x:c r="B63" s="18" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C63" s="6" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="D63" s="6" t="str">
+        <x:v>Requisito heredado</x:v>
+      </x:c>
+      <x:c r="E63" s="6" t="str">
+        <x:v>ET-03</x:v>
+      </x:c>
+      <x:c r="F63" s="6" t="str">
+        <x:v>Área compartida central y comunicaciones</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="50" customHeight="1">
+      <x:c r="A64" s="6" t="str">
+        <x:v>Buffers RAW para estimación</x:v>
+      </x:c>
+      <x:c r="B64" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C64" s="6" t="str">
+        <x:v>buffers</x:v>
+      </x:c>
+      <x:c r="D64" s="6" t="str">
+        <x:v>Criterio aprobado</x:v>
+      </x:c>
+      <x:c r="E64" s="6" t="str">
+        <x:v>SEL-002</x:v>
+      </x:c>
+      <x:c r="F64" s="6" t="str">
+        <x:v>No dimensiona RAM total de Linux y aplicación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="30" customHeight="1">
+      <x:c r="A67" s="6" t="str">
+        <x:v>SRC-009</x:v>
+      </x:c>
+      <x:c r="B67" s="6" t="str">
+        <x:v>Toradex Verdin V1.1 datasheet rev.1.8; tablas 7, 51–53 y 72</x:v>
+      </x:c>
+      <x:c r="C67" s="6"/>
+      <x:c r="D67" s="6"/>
+      <x:c r="E67" s="6"/>
+      <x:c r="F67" s="6"/>
+    </x:row>
+    <x:row r="68" ht="42" customHeight="1">
+      <x:c r="A68" s="6" t="str">
+        <x:v>https://docs.toradex.com/116795-verdin_imx8mp_datasheet.pdf</x:v>
+      </x:c>
+      <x:c r="B68" s="6"/>
+      <x:c r="C68" s="6"/>
+      <x:c r="D68" s="6"/>
+      <x:c r="E68" s="6"/>
+      <x:c r="F68" s="6"/>
+    </x:row>
+    <x:row r="69" ht="30" customHeight="1">
+      <x:c r="A69" s="6"/>
+      <x:c r="B69" s="6"/>
+      <x:c r="C69" s="6"/>
+      <x:c r="D69" s="6"/>
+      <x:c r="E69" s="6"/>
+      <x:c r="F69" s="6"/>
+    </x:row>
+    <x:row r="70" ht="30" customHeight="1">
+      <x:c r="A70" s="6" t="str">
+        <x:v>SRC-010</x:v>
+      </x:c>
+      <x:c r="B70" s="6" t="str">
+        <x:v>Toradex PCN 0063: reemplazo V1.1A por V1.1B</x:v>
+      </x:c>
+      <x:c r="C70" s="6"/>
+      <x:c r="D70" s="6"/>
+      <x:c r="E70" s="6"/>
+      <x:c r="F70" s="6"/>
+    </x:row>
+    <x:row r="71" ht="42" customHeight="1">
+      <x:c r="A71" s="6" t="str">
+        <x:v>https://docs.toradex.com/114344-pcn-0063-v11a-v11b-20231127.pdf</x:v>
+      </x:c>
+      <x:c r="B71" s="6"/>
+      <x:c r="C71" s="6"/>
+      <x:c r="D71" s="6"/>
+      <x:c r="E71" s="6"/>
+      <x:c r="F71" s="6"/>
+    </x:row>
+    <x:row r="72" ht="30" customHeight="1">
+      <x:c r="A72" s="6"/>
+      <x:c r="B72" s="6"/>
+      <x:c r="C72" s="6"/>
+      <x:c r="D72" s="6"/>
+      <x:c r="E72" s="6"/>
+      <x:c r="F72" s="6"/>
+    </x:row>
+    <x:row r="73" ht="30" customHeight="1">
+      <x:c r="A73" s="6" t="str">
+        <x:v>SRC-011</x:v>
+      </x:c>
+      <x:c r="B73" s="6" t="str">
+        <x:v>Verdin Carrier Board Design Guide V1.2; §3.1 alimentación</x:v>
+      </x:c>
+      <x:c r="C73" s="6"/>
+      <x:c r="D73" s="6"/>
+      <x:c r="E73" s="6"/>
+      <x:c r="F73" s="6"/>
+    </x:row>
+    <x:row r="74" ht="42" customHeight="1">
+      <x:c r="A74" s="6" t="str">
+        <x:v>https://docs.toradex.com/108140-verdin-carrier-board-design-guide.pdf</x:v>
+      </x:c>
+      <x:c r="B74" s="6"/>
+      <x:c r="C74" s="6"/>
+      <x:c r="D74" s="6"/>
+      <x:c r="E74" s="6"/>
+      <x:c r="F74" s="6"/>
+    </x:row>
+    <x:row r="75" ht="30" customHeight="1">
+      <x:c r="A75" s="6"/>
+      <x:c r="B75" s="6"/>
+      <x:c r="C75" s="6"/>
+      <x:c r="D75" s="6"/>
+      <x:c r="E75" s="6"/>
+      <x:c r="F75" s="6"/>
+    </x:row>
+    <x:row r="76" ht="30" customHeight="1">
+      <x:c r="A76" s="6" t="str">
+        <x:v>SRC-012</x:v>
+      </x:c>
+      <x:c r="B76" s="6" t="str">
+        <x:v>Kingston SDCIT2, 2 páginas; capacidades, referencias y límites publicados</x:v>
+      </x:c>
+      <x:c r="C76" s="6"/>
+      <x:c r="D76" s="6"/>
+      <x:c r="E76" s="6"/>
+      <x:c r="F76" s="6"/>
+    </x:row>
+    <x:row r="77" ht="42" customHeight="1">
+      <x:c r="A77" s="6" t="str">
+        <x:v>https://www.kingston.com/datasheets/sdcit2_en.pdf</x:v>
+      </x:c>
+      <x:c r="B77" s="6"/>
+      <x:c r="C77" s="6"/>
+      <x:c r="D77" s="6"/>
+      <x:c r="E77" s="6"/>
+      <x:c r="F77" s="6"/>
+    </x:row>
+    <x:row r="78" ht="30" customHeight="1">
+      <x:c r="A78" s="6"/>
+      <x:c r="B78" s="6"/>
+      <x:c r="C78" s="6"/>
+      <x:c r="D78" s="6"/>
+      <x:c r="E78" s="6"/>
+      <x:c r="F78" s="6"/>
+    </x:row>
+    <x:row r="79" ht="30" customHeight="1">
+      <x:c r="A79" s="6" t="str">
+        <x:v>SRC-013</x:v>
+      </x:c>
+      <x:c r="B79" s="6" t="str">
+        <x:v>Toradex SD/MMC Card (Linux); ejemplo Verdin iMX8M Plus</x:v>
+      </x:c>
+      <x:c r="C79" s="6"/>
+      <x:c r="D79" s="6"/>
+      <x:c r="E79" s="6"/>
+      <x:c r="F79" s="6"/>
+    </x:row>
+    <x:row r="80" ht="42" customHeight="1">
+      <x:c r="A80" s="6" t="str">
+        <x:v>https://developer.toradex.com/linux-bsp/application-development/peripheral-access/sdmmc-card-linux/</x:v>
+      </x:c>
+      <x:c r="B80" s="6"/>
+      <x:c r="C80" s="6"/>
+      <x:c r="D80" s="6"/>
+      <x:c r="E80" s="6"/>
+      <x:c r="F80" s="6"/>
+    </x:row>
+    <x:row r="81" ht="30" customHeight="1">
+      <x:c r="A81" s="6"/>
+      <x:c r="B81" s="6"/>
+      <x:c r="C81" s="6"/>
+      <x:c r="D81" s="6"/>
+      <x:c r="E81" s="6"/>
+      <x:c r="F81" s="6"/>
+    </x:row>
+    <x:row r="82" ht="30" customHeight="1">
+      <x:c r="A82" s="6"/>
+      <x:c r="B82" s="6"/>
+      <x:c r="C82" s="6"/>
+      <x:c r="D82" s="6"/>
+      <x:c r="E82" s="6"/>
+      <x:c r="F82" s="6"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1462,6 +2587,16 @@
     <x:mergeCell ref="A38:F38"/>
     <x:mergeCell ref="B40:F40"/>
     <x:mergeCell ref="A41:F41"/>
+    <x:mergeCell ref="B67:F67"/>
+    <x:mergeCell ref="A68:F68"/>
+    <x:mergeCell ref="B70:F70"/>
+    <x:mergeCell ref="A71:F71"/>
+    <x:mergeCell ref="B73:F73"/>
+    <x:mergeCell ref="A74:F74"/>
+    <x:mergeCell ref="B76:F76"/>
+    <x:mergeCell ref="A77:F77"/>
+    <x:mergeCell ref="B79:F79"/>
+    <x:mergeCell ref="A80:F80"/>
   </x:mergeCells>
   <x:dataValidations count="8">
     <x:dataValidation type="list" sqref="B9">
@@ -1579,7 +2714,7 @@
         <x:v>Esquemático y compatibilidad de controlador, SDK y sistema.</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
-        <x:v>Pendiente de computador</x:v>
+        <x:v>Verdin adoptado; SDK por validar</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="86" customHeight="1">
@@ -1662,21 +2797,85 @@
         <x:v>Pendiente de implementación</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="26" customHeight="1">
-      <x:c r="A11" s="2"/>
-      <x:c r="B11" s="2"/>
-      <x:c r="C11" s="2"/>
-      <x:c r="D11" s="2"/>
-      <x:c r="E11" s="2"/>
-      <x:c r="F11" s="2"/>
-    </x:row>
-    <x:row r="12" ht="26" customHeight="1">
-      <x:c r="A12" s="2"/>
-      <x:c r="B12" s="2"/>
-      <x:c r="C12" s="2"/>
-      <x:c r="D12" s="2"/>
-      <x:c r="E12" s="2"/>
-      <x:c r="F12" s="2"/>
+    <x:row r="11" ht="86" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>PCB-06</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>ET-04; IF-09</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>microSD industrial independiente; mantener eMMC para arranque.</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>SEL-003; SRC-012/013</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>Capacidad útil ≥15 GB; 90 días según cuotas.</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Capacidad real por verificar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="86" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>PCB-07</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>IF-09; ET-02</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>SD de 4 bits, 25 MHz y señalización 3,3 V.</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>SRC-009 §5.14</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>SD_1_PWR_EN es 1,8 V; revisar EN y pull-ups.</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Zócalo y circuito por elegir</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="86" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>PCB-08</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>IF-09; integridad</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>No cortar energía con escrituras activas; retener tarjeta.</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Criterio de diseño; SRC-012</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>Protección publicada no garantiza último archivo.</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Corriente pico y arranque pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="86" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>PCB-09</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>ET-02; SEL-002</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>Rama SoM 5 V ±5 % en VCC, capacidad 3 A.</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>SRC-011 §3.1; cálculo</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>Verificar caída, rampa y transitorios. Excluye otras cargas.</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>Circuito por implementar</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
design: integrar contratos de interfaces entre modulos
</commit_message>
<xml_diff>
--- a/calculos/calculos_y_restricciones.xlsx
+++ b/calculos/calculos_y_restricciones.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="R928caf0751474268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="Rb236232de79e4305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rd7c633aaad2945d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="Rda207b0494c346f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="R3099d58c8b434b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rfd52b1bb5f0044bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -44,7 +44,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,6 +71,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -84,7 +89,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -144,6 +149,12 @@
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -154,7 +165,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -164,7 +175,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1354,10 +1365,42 @@
       <x:c r="D74" s="6"/>
     </x:row>
     <x:row r="75" ht="34" customHeight="1">
-      <x:c r="A75" s="6"/>
+      <x:c r="A75" s="6" t="str">
+        <x:v>UART de actitud: techo antes de protocolo</x:v>
+      </x:c>
       <x:c r="B75" s="6"/>
       <x:c r="C75" s="6"/>
       <x:c r="D75" s="6"/>
+    </x:row>
+    <x:row r="76" ht="34" customHeight="1">
+      <x:c r="A76" s="6" t="str">
+        <x:v>Bits transmitidos por byte</x:v>
+      </x:c>
+      <x:c r="B76" s="20" t="n">
+        <x:f>SUM('Entradas'!B85:B87)</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C76" s="6" t="str">
+        <x:v>bits</x:v>
+      </x:c>
+      <x:c r="D76" s="6" t="str">
+        <x:v>Inicio + datos + parada; 8N1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="34" customHeight="1">
+      <x:c r="A77" s="6" t="str">
+        <x:v>Techo de carga útil UART</x:v>
+      </x:c>
+      <x:c r="B77" s="20" t="n">
+        <x:f>'Entradas'!B84/B76</x:f>
+        <x:v>11520</x:v>
+      </x:c>
+      <x:c r="C77" s="6" t="str">
+        <x:v>bytes/s</x:v>
+      </x:c>
+      <x:c r="D77" s="6" t="str">
+        <x:v>No acredita suficiencia de telemetría ni descuenta cabeceras.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B45:B45">
@@ -2576,6 +2619,106 @@
       <x:c r="D82" s="6"/>
       <x:c r="E82" s="6"/>
       <x:c r="F82" s="6"/>
+    </x:row>
+    <x:row r="84" ht="50" customHeight="1">
+      <x:c r="A84" s="6" t="str">
+        <x:v>Contrato de actitud: UART</x:v>
+      </x:c>
+      <x:c r="B84" s="22" t="n">
+        <x:v>115200</x:v>
+      </x:c>
+      <x:c r="C84" s="6" t="str">
+        <x:v>bit/s</x:v>
+      </x:c>
+      <x:c r="D84" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E84" s="6" t="str">
+        <x:v>Contrato interfaces</x:v>
+      </x:c>
+      <x:c r="F84" s="6" t="str">
+        <x:v>Controlador ADCS externo; 8N1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="50" customHeight="1">
+      <x:c r="A85" s="6" t="str">
+        <x:v>Bits de inicio por carácter</x:v>
+      </x:c>
+      <x:c r="B85" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C85" s="6" t="str">
+        <x:v>bit</x:v>
+      </x:c>
+      <x:c r="D85" s="6" t="str">
+        <x:v>Formato 8N1</x:v>
+      </x:c>
+      <x:c r="E85" s="6" t="str">
+        <x:v>Contrato interfaces</x:v>
+      </x:c>
+      <x:c r="F85" s="6" t="str">
+        <x:v>Sin paridad</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="50" customHeight="1">
+      <x:c r="A86" s="6" t="str">
+        <x:v>Bits de datos por carácter</x:v>
+      </x:c>
+      <x:c r="B86" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C86" s="6" t="str">
+        <x:v>bits</x:v>
+      </x:c>
+      <x:c r="D86" s="6" t="str">
+        <x:v>Formato 8N1</x:v>
+      </x:c>
+      <x:c r="E86" s="6" t="str">
+        <x:v>Contrato interfaces</x:v>
+      </x:c>
+      <x:c r="F86" s="6" t="str">
+        <x:v>Un byte de carga por carácter</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="50" customHeight="1">
+      <x:c r="A87" s="6" t="str">
+        <x:v>Bits de parada por carácter</x:v>
+      </x:c>
+      <x:c r="B87" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C87" s="6" t="str">
+        <x:v>bit</x:v>
+      </x:c>
+      <x:c r="D87" s="6" t="str">
+        <x:v>Formato 8N1</x:v>
+      </x:c>
+      <x:c r="E87" s="6" t="str">
+        <x:v>Contrato interfaces</x:v>
+      </x:c>
+      <x:c r="F87" s="6" t="str">
+        <x:v>No incluye cabeceras de trama</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="50" customHeight="1">
+      <x:c r="A88" s="6" t="str">
+        <x:v>Reloj I2C hacia EPS</x:v>
+      </x:c>
+      <x:c r="B88" s="22" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C88" s="6" t="str">
+        <x:v>kHz</x:v>
+      </x:c>
+      <x:c r="D88" s="6" t="str">
+        <x:v>Diseño aprobado</x:v>
+      </x:c>
+      <x:c r="E88" s="6" t="str">
+        <x:v>Contrato interfaces</x:v>
+      </x:c>
+      <x:c r="F88" s="6" t="str">
+        <x:v>Dirección y presupuesto de capacitancia por cerrar</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2745,16 +2888,16 @@
         <x:v>IF-02; ET-02</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
-        <x:v>Dimensionar alimentación de cámara por consumo máximo y arranque.</x:v>
+        <x:v>Cámara alimentada por el conjunto externo; definir VBUS y retorno.</x:v>
       </x:c>
       <x:c r="D8" s="6" t="str">
-        <x:v>SRC-001 solo publica 1,6 W; máximo pendiente</x:v>
+        <x:v>SRC-002 y contrato aprobado de interfaces</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
-        <x:v>Cálculo de corriente, protección, caída y secuencia.</x:v>
+        <x:v>Evitar retroalimentación; no eliminar VBUS ni unir fuentes sin diseño.</x:v>
       </x:c>
       <x:c r="F8" s="6" t="str">
-        <x:v>No usar 0,32 A como máximo</x:v>
+        <x:v>Topología física externa por cerrar</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="86" customHeight="1">
@@ -2875,6 +3018,86 @@
       </x:c>
       <x:c r="F14" s="6" t="str">
         <x:v>Circuito por implementar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="86" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>PCB-10</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>IF-16</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>I2C_1 a EPS: 100 kHz; PGOOD y ALERT_N.</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>Contrato aprobado; SRC-009</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>Dominio externo 3,3 V; adaptación I2C, pull-ups y estados.</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>Pines GPIO y componentes pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="86" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>PCB-11</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>IF-14/15</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>UART_1 a controlador ADCS externo: 115200 bit/s, 8N1.</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Contrato aprobado; SRC-009</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>3,3 V externos, TX a RX, masa común y tramas.</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>Carga de datos y temporización pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="86" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>PCB-12</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>IF-10/11</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>SPI_1 interno; Verdin maestro; cuatro señales.</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>Acuerdo comunicaciones; SRC-009</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>MOSI/SCK/CS salen; MISO entra. Validar niveles del receptor.</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>Modo y frecuencia pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="86" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>PCB-13</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>IF-C01</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>USB_1 recuperación y UART_3 consola.</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>SRC-009; contrato aprobado</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="str">
+        <x:v>Referencias reales de tensión; no confundir referencia con alimentación.</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>Conectores y secuencia por definir</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
design: integrar adaptacion UART y calculos de polarizacion
</commit_message>
<xml_diff>
--- a/calculos/calculos_y_restricciones.xlsx
+++ b/calculos/calculos_y_restricciones.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="Rda207b0494c346f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="R3099d58c8b434b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rfd52b1bb5f0044bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="R76af41dae72a434a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="R8e47d6f010844a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rbb34f11d8c7f4292"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,11 +15,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000"/>
     <x:numFmt numFmtId="203" formatCode="#,##0"/>
+    <x:numFmt numFmtId="204" formatCode="0.###"/>
+    <x:numFmt numFmtId="205" formatCode="0%"/>
+    <x:numFmt numFmtId="206" formatCode="0.0000"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -44,7 +47,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +79,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -89,7 +97,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -153,6 +161,18 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1402,6 +1422,121 @@
         <x:v>No acredita suficiencia de telemetría ni descuenta cabeceras.</x:v>
       </x:c>
     </x:row>
+    <x:row r="79" ht="44" customHeight="1">
+      <x:c r="A79" s="6" t="str">
+        <x:v>Polarización UART: cotas por resistencia</x:v>
+      </x:c>
+      <x:c r="B79" s="6"/>
+      <x:c r="C79" s="6"/>
+      <x:c r="D79" s="6" t="str">
+        <x:v>No representa consumo total ni permanente de la interfaz.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="44" customHeight="1">
+      <x:c r="A80" s="6" t="str">
+        <x:v>Resistencia mínima</x:v>
+      </x:c>
+      <x:c r="B80" s="20" t="n">
+        <x:f>'Entradas'!B90*(1-'Entradas'!B91)</x:f>
+        <x:v>9900</x:v>
+      </x:c>
+      <x:c r="C80" s="6" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="D80" s="6" t="str">
+        <x:v>Valor nominal menos tolerancia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="44" customHeight="1">
+      <x:c r="A81" s="6" t="str">
+        <x:v>Resistencia máxima</x:v>
+      </x:c>
+      <x:c r="B81" s="20" t="n">
+        <x:f>'Entradas'!B90*(1+'Entradas'!B91)</x:f>
+        <x:v>10100</x:v>
+      </x:c>
+      <x:c r="C81" s="6" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="D81" s="6" t="str">
+        <x:v>Valor nominal más tolerancia.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="44" customHeight="1">
+      <x:c r="A82" s="6" t="str">
+        <x:v>Corriente máxima por resistencia A</x:v>
+      </x:c>
+      <x:c r="B82" s="26" t="n">
+        <x:f>'Entradas'!B92/B80*1000</x:f>
+        <x:v>0.19696969696969696</x:v>
+      </x:c>
+      <x:c r="C82" s="6" t="str">
+        <x:v>mA</x:v>
+      </x:c>
+      <x:c r="D82" s="6" t="str">
+        <x:v>Cuando soporta toda la tensión de 1,95 V.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="44" customHeight="1">
+      <x:c r="A83" s="6" t="str">
+        <x:v>Corriente máxima por resistencia B</x:v>
+      </x:c>
+      <x:c r="B83" s="26" t="n">
+        <x:f>'Entradas'!B93/B80*1000</x:f>
+        <x:v>0.36363636363636365</x:v>
+      </x:c>
+      <x:c r="C83" s="6" t="str">
+        <x:v>mA</x:v>
+      </x:c>
+      <x:c r="D83" s="6" t="str">
+        <x:v>Cuando soporta toda la tensión de 3,6 V.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="44" customHeight="1">
+      <x:c r="A84" s="6" t="str">
+        <x:v>Potencia máxima por resistencia A</x:v>
+      </x:c>
+      <x:c r="B84" s="26" t="n">
+        <x:f>'Entradas'!B92^2/B80*1000</x:f>
+        <x:v>0.3840909090909091</x:v>
+      </x:c>
+      <x:c r="C84" s="6" t="str">
+        <x:v>mW</x:v>
+      </x:c>
+      <x:c r="D84" s="6" t="str">
+        <x:v>V²/R; verificar derating del componente elegido.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="44" customHeight="1">
+      <x:c r="A85" s="6" t="str">
+        <x:v>Potencia máxima por resistencia B</x:v>
+      </x:c>
+      <x:c r="B85" s="26" t="n">
+        <x:f>'Entradas'!B93^2/B80*1000</x:f>
+        <x:v>1.3090909090909093</x:v>
+      </x:c>
+      <x:c r="C85" s="6" t="str">
+        <x:v>mW</x:v>
+      </x:c>
+      <x:c r="D85" s="6" t="str">
+        <x:v>V²/R; no equivale a potencia del traductor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="44" customHeight="1">
+      <x:c r="A86" s="6" t="str">
+        <x:v>Caída/cota por fuga reservada</x:v>
+      </x:c>
+      <x:c r="B86" s="26" t="n">
+        <x:f>SUM('Entradas'!B94:B95)/1000000*B81</x:f>
+        <x:v>0.1212</x:v>
+      </x:c>
+      <x:c r="C86" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D86" s="6" t="str">
+        <x:v>OE en alta impedancia o caída en pull-up; umbrales por comprobar.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="B45:B45">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
@@ -2718,6 +2853,166 @@
       </x:c>
       <x:c r="F88" s="6" t="str">
         <x:v>Dirección y presupuesto de capacitancia por cerrar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="60" customHeight="1">
+      <x:c r="A90" s="6" t="str">
+        <x:v>Resistencia de polarización UART</x:v>
+      </x:c>
+      <x:c r="B90" s="24" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="C90" s="6" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="D90" s="6" t="str">
+        <x:v>Decisión aprobada</x:v>
+      </x:c>
+      <x:c r="E90" s="6" t="str">
+        <x:v>SEL-004</x:v>
+      </x:c>
+      <x:c r="F90" s="6" t="str">
+        <x:v>Tres pull-ups; un pull-down de OE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="60" customHeight="1">
+      <x:c r="A91" s="6" t="str">
+        <x:v>Tolerancia de resistencias</x:v>
+      </x:c>
+      <x:c r="B91" s="25" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C91" s="6" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="D91" s="6" t="str">
+        <x:v>Decisión aprobada</x:v>
+      </x:c>
+      <x:c r="E91" s="6" t="str">
+        <x:v>SEL-004</x:v>
+      </x:c>
+      <x:c r="F91" s="6" t="str">
+        <x:v>1 %; no incluye variación térmica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="60" customHeight="1">
+      <x:c r="A92" s="6" t="str">
+        <x:v>Envolvente A: tensión máxima</x:v>
+      </x:c>
+      <x:c r="B92" s="24" t="n">
+        <x:v>1.95</x:v>
+      </x:c>
+      <x:c r="C92" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D92" s="6" t="str">
+        <x:v>Hipótesis de evaluación</x:v>
+      </x:c>
+      <x:c r="E92" s="6" t="str">
+        <x:v>SEL-004</x:v>
+      </x:c>
+      <x:c r="F92" s="6" t="str">
+        <x:v>Riel real debe quedar contenido en 1,65–1,95 V</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="60" customHeight="1">
+      <x:c r="A93" s="6" t="str">
+        <x:v>Envolvente B: tensión máxima</x:v>
+      </x:c>
+      <x:c r="B93" s="24" t="n">
+        <x:v>3.6</x:v>
+      </x:c>
+      <x:c r="C93" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D93" s="6" t="str">
+        <x:v>Hipótesis de evaluación</x:v>
+      </x:c>
+      <x:c r="E93" s="6" t="str">
+        <x:v>SEL-004</x:v>
+      </x:c>
+      <x:c r="F93" s="6" t="str">
+        <x:v>Riel real debe quedar contenido en 3,0–3,6 V</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="60" customHeight="1">
+      <x:c r="A94" s="6" t="str">
+        <x:v>Fuga adicional por extremo</x:v>
+      </x:c>
+      <x:c r="B94" s="24" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C94" s="6" t="str">
+        <x:v>uA</x:v>
+      </x:c>
+      <x:c r="D94" s="6" t="str">
+        <x:v>Requisito; por verificar</x:v>
+      </x:c>
+      <x:c r="E94" s="6" t="str">
+        <x:v>SEL-004</x:v>
+      </x:c>
+      <x:c r="F94" s="6" t="str">
+        <x:v>No es dato medido del GPIO o módulo externo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="60" customHeight="1">
+      <x:c r="A95" s="6" t="str">
+        <x:v>Fuga de entrada del traductor</x:v>
+      </x:c>
+      <x:c r="B95" s="24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C95" s="6" t="str">
+        <x:v>uA</x:v>
+      </x:c>
+      <x:c r="D95" s="6" t="str">
+        <x:v>Dato del fabricante</x:v>
+      </x:c>
+      <x:c r="E95" s="6" t="str">
+        <x:v>SRC-014; §7.3/7.5</x:v>
+      </x:c>
+      <x:c r="F95" s="6" t="str">
+        <x:v>Incluye polarización interna; rango térmico completo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="60" customHeight="1">
+      <x:c r="A96" s="6" t="str">
+        <x:v>Desacoplo por alimentación</x:v>
+      </x:c>
+      <x:c r="B96" s="24" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C96" s="6" t="str">
+        <x:v>nF</x:v>
+      </x:c>
+      <x:c r="D96" s="6" t="str">
+        <x:v>Recomendación fabricante</x:v>
+      </x:c>
+      <x:c r="E96" s="6" t="str">
+        <x:v>SRC-014; §12.1</x:v>
+      </x:c>
+      <x:c r="F96" s="6" t="str">
+        <x:v>Dos condensadores; referencia exacta por seleccionar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="60" customHeight="1">
+      <x:c r="A97" s="6" t="str">
+        <x:v>Potencia nominal mínima resistencia</x:v>
+      </x:c>
+      <x:c r="B97" s="24" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="C97" s="6" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="D97" s="6" t="str">
+        <x:v>Decisión de diseño</x:v>
+      </x:c>
+      <x:c r="E97" s="6" t="str">
+        <x:v>SEL-004</x:v>
+      </x:c>
+      <x:c r="F97" s="6" t="str">
+        <x:v>Comprobar reducción de potencia con temperatura</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3100,6 +3395,46 @@
         <x:v>Conectores y secuencia por definir</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="95" customHeight="1">
+      <x:c r="A19" s="6" t="str">
+        <x:v>PCB-14</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="str">
+        <x:v>IF-14/15; SEL-004</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="str">
+        <x:v>TXU0202: desacoplo de 100 nF por fuente, junto a sus pines.</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="str">
+        <x:v>SRC-014 §12.1; recomendación adoptada</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="str">
+        <x:v>Retornos cortos; revisar flancos, carga y referencias de alimentación.</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="str">
+        <x:v>Ubicación, GPIO OE y ESD pendientes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="95" customHeight="1">
+      <x:c r="A20" s="6" t="str">
+        <x:v>PCB-15</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="str">
+        <x:v>IF-14/15; SEL-004</x:v>
+      </x:c>
+      <x:c r="C20" s="6" t="str">
+        <x:v>ADCS apagado: tolerar señales hasta 3,6 V y fuga ≤10 uA por pin.</x:v>
+      </x:c>
+      <x:c r="D20" s="6" t="str">
+        <x:v>Contrato externo aprobado; SRC-014 §9.3 para límites del traductor</x:v>
+      </x:c>
+      <x:c r="E20" s="6" t="str">
+        <x:v>Verificar aislamiento remoto; OE local no detecta por sí solo apagado remoto.</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="str">
+        <x:v>Requisito externo; no validado físicamente</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
design: publicar UART para captura inicial y revision electrica
</commit_message>
<xml_diff>
--- a/calculos/calculos_y_restricciones.xlsx
+++ b/calculos/calculos_y_restricciones.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="R76af41dae72a434a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="R8e47d6f010844a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rbb34f11d8c7f4292"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculos" sheetId="1" r:id="R3e4d54e41ae942ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entradas" sheetId="2" r:id="R01d08934f9c34de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Restricciones" sheetId="3" r:id="Rb52e9c5e6b404f84"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000"/>
@@ -23,6 +23,7 @@
     <x:numFmt numFmtId="204" formatCode="0.###"/>
     <x:numFmt numFmtId="205" formatCode="0%"/>
     <x:numFmt numFmtId="206" formatCode="0.0000"/>
+    <x:numFmt numFmtId="207" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -47,7 +48,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -84,6 +85,11 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -97,7 +103,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -173,6 +179,15 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1436,30 +1451,30 @@
       <x:c r="A80" s="6" t="str">
         <x:v>Resistencia mínima</x:v>
       </x:c>
-      <x:c r="B80" s="20" t="n">
-        <x:f>'Entradas'!B90*(1-'Entradas'!B91)</x:f>
-        <x:v>9900</x:v>
+      <x:c r="B80" s="29" t="n">
+        <x:f>'Entradas'!B90*(1-'Entradas'!B91)*(1-'Entradas'!B99/1000000*'Entradas'!B100)</x:f>
+        <x:v>9835.65</x:v>
       </x:c>
       <x:c r="C80" s="6" t="str">
         <x:v>ohm</x:v>
       </x:c>
       <x:c r="D80" s="6" t="str">
-        <x:v>Valor nominal menos tolerancia.</x:v>
+        <x:v>10 kohm: tolerancia inicial y coeficiente térmico.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="44" customHeight="1">
       <x:c r="A81" s="6" t="str">
         <x:v>Resistencia máxima</x:v>
       </x:c>
-      <x:c r="B81" s="20" t="n">
-        <x:f>'Entradas'!B90*(1+'Entradas'!B91)</x:f>
-        <x:v>10100</x:v>
+      <x:c r="B81" s="29" t="n">
+        <x:f>'Entradas'!B90*(1+'Entradas'!B91)*(1+'Entradas'!B99/1000000*'Entradas'!B100)</x:f>
+        <x:v>10165.65</x:v>
       </x:c>
       <x:c r="C81" s="6" t="str">
         <x:v>ohm</x:v>
       </x:c>
       <x:c r="D81" s="6" t="str">
-        <x:v>Valor nominal más tolerancia.</x:v>
+        <x:v>10 kohm: tolerancia inicial y coeficiente térmico.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="44" customHeight="1">
@@ -1468,7 +1483,7 @@
       </x:c>
       <x:c r="B82" s="26" t="n">
         <x:f>'Entradas'!B92/B80*1000</x:f>
-        <x:v>0.19696969696969696</x:v>
+        <x:v>0.1982583764164036</x:v>
       </x:c>
       <x:c r="C82" s="6" t="str">
         <x:v>mA</x:v>
@@ -1483,7 +1498,7 @@
       </x:c>
       <x:c r="B83" s="26" t="n">
         <x:f>'Entradas'!B93/B80*1000</x:f>
-        <x:v>0.36363636363636365</x:v>
+        <x:v>0.3660154641533605</x:v>
       </x:c>
       <x:c r="C83" s="6" t="str">
         <x:v>mA</x:v>
@@ -1498,7 +1513,7 @@
       </x:c>
       <x:c r="B84" s="26" t="n">
         <x:f>'Entradas'!B92^2/B80*1000</x:f>
-        <x:v>0.3840909090909091</x:v>
+        <x:v>0.386603834011987</x:v>
       </x:c>
       <x:c r="C84" s="6" t="str">
         <x:v>mW</x:v>
@@ -1513,7 +1528,7 @@
       </x:c>
       <x:c r="B85" s="26" t="n">
         <x:f>'Entradas'!B93^2/B80*1000</x:f>
-        <x:v>1.3090909090909093</x:v>
+        <x:v>1.317655670952098</x:v>
       </x:c>
       <x:c r="C85" s="6" t="str">
         <x:v>mW</x:v>
@@ -1524,17 +1539,167 @@
     </x:row>
     <x:row r="86" ht="44" customHeight="1">
       <x:c r="A86" s="6" t="str">
-        <x:v>Caída/cota por fuga reservada</x:v>
+        <x:v>Cota de OE deshabilitado por fuga</x:v>
       </x:c>
       <x:c r="B86" s="26" t="n">
-        <x:f>SUM('Entradas'!B94:B95)/1000000*B81</x:f>
-        <x:v>0.1212</x:v>
+        <x:f>('Entradas'!B102+'Entradas'!B95)/1000000*B81</x:f>
+        <x:v>0.0609939</x:v>
       </x:c>
       <x:c r="C86" s="6" t="str">
         <x:v>V</x:v>
       </x:c>
       <x:c r="D86" s="6" t="str">
-        <x:v>OE en alta impedancia o caída en pull-up; umbrales por comprobar.</x:v>
+        <x:v>GPIO en alta impedancia: 4 uA NXP + 2 uA TI; no salida activa.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="48" customHeight="1">
+      <x:c r="A88" s="6" t="str">
+        <x:v>Resistencia mínima A2Y</x:v>
+      </x:c>
+      <x:c r="B88" s="26" t="n">
+        <x:f>'Entradas'!B98*(1-'Entradas'!B91)*(1-'Entradas'!B99/1000000*'Entradas'!B100)</x:f>
+        <x:v>46227.555</x:v>
+      </x:c>
+      <x:c r="C88" s="6" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="D88" s="6" t="str">
+        <x:v>47 kohm con tolerancia y temperatura.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="48" customHeight="1">
+      <x:c r="A89" s="6" t="str">
+        <x:v>Resistencia máxima A2Y</x:v>
+      </x:c>
+      <x:c r="B89" s="26" t="n">
+        <x:f>'Entradas'!B98*(1+'Entradas'!B91)*(1+'Entradas'!B99/1000000*'Entradas'!B100)</x:f>
+        <x:v>47778.555</x:v>
+      </x:c>
+      <x:c r="C89" s="6" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="D89" s="6" t="str">
+        <x:v>47 kohm con tolerancia y temperatura.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="48" customHeight="1">
+      <x:c r="A90" s="6" t="str">
+        <x:v>Carga estática máxima A2Y</x:v>
+      </x:c>
+      <x:c r="B90" s="26" t="n">
+        <x:f>'Entradas'!B92/B88*1000000+'Entradas'!B102</x:f>
+        <x:v>46.182633280085874</x:v>
+      </x:c>
+      <x:c r="C90" s="6" t="str">
+        <x:v>uA</x:v>
+      </x:c>
+      <x:c r="D90" s="6" t="str">
+        <x:v>Debe ser ≤100 uA para usar VOH=VCC−0,1 y VOL=0,1 V.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="48" customHeight="1">
+      <x:c r="A91" s="6" t="str">
+        <x:v>Carga estática máxima B1Y</x:v>
+      </x:c>
+      <x:c r="B91" s="26" t="n">
+        <x:f>'Entradas'!B93/B88*1000000+'Entradas'!B94+'Entradas'!B103</x:f>
+        <x:v>87.92563067092776</x:v>
+      </x:c>
+      <x:c r="C91" s="6" t="str">
+        <x:v>uA</x:v>
+      </x:c>
+      <x:c r="D91" s="6" t="str">
+        <x:v>Pull-up externo 47 kohm con igual envolvente; fuga externa y TVS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="48" customHeight="1">
+      <x:c r="A92" s="6" t="str">
+        <x:v>Margen alto: traductor → Verdin</x:v>
+      </x:c>
+      <x:c r="B92" s="26" t="n">
+        <x:f>'Entradas'!B101-0.1-'Entradas'!B104*'Entradas'!B92</x:f>
+        <x:v>0.18499999999999983</x:v>
+      </x:c>
+      <x:c r="C92" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D92" s="6" t="str">
+        <x:v>No valida dirección Verdin → traductor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="48" customHeight="1">
+      <x:c r="A93" s="6" t="str">
+        <x:v>Margen bajo: traductor → Verdin</x:v>
+      </x:c>
+      <x:c r="B93" s="26" t="n">
+        <x:f>'Entradas'!B105*'Entradas'!B101-0.1</x:f>
+        <x:v>0.3949999999999999</x:v>
+      </x:c>
+      <x:c r="C93" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D93" s="6" t="str">
+        <x:v>Extremos independientes de alimentación; carga indicada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="48" customHeight="1">
+      <x:c r="A94" s="6" t="str">
+        <x:v>Margen alto: traductor → ADCS</x:v>
+      </x:c>
+      <x:c r="B94" s="26" t="n">
+        <x:f>3-0.1-'Entradas'!B106</x:f>
+        <x:v>0.3799999999999999</x:v>
+      </x:c>
+      <x:c r="C94" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D94" s="6" t="str">
+        <x:v>VCCB mínimo 3,0 V; receptor externo definido por contrato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="48" customHeight="1">
+      <x:c r="A95" s="6" t="str">
+        <x:v>Margen bajo: traductor → ADCS</x:v>
+      </x:c>
+      <x:c r="B95" s="26" t="n">
+        <x:f>'Entradas'!B107-0.1</x:f>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="C95" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D95" s="6" t="str">
+        <x:v>Receptor externo definido por contrato.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="48" customHeight="1">
+      <x:c r="A96" s="6" t="str">
+        <x:v>Cota estática conservadora lado A</x:v>
+      </x:c>
+      <x:c r="B96" s="26" t="n">
+        <x:f>2*B82+'Entradas'!B92/B88*1000+0.006</x:f>
+        <x:v>0.44469938611289306</x:v>
+      </x:c>
+      <x:c r="C96" s="6" t="str">
+        <x:v>mA</x:v>
+      </x:c>
+      <x:c r="D96" s="6" t="str">
+        <x:v>Incluye polarización y 6 uA del traductor; excluye dinámica.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="48" customHeight="1">
+      <x:c r="A97" s="6" t="str">
+        <x:v>Potencia máxima pull-up A2Y</x:v>
+      </x:c>
+      <x:c r="B97" s="26" t="n">
+        <x:f>'Entradas'!B92^2/B88*1000</x:f>
+        <x:v>0.08225613489616744</x:v>
+      </x:c>
+      <x:c r="C97" s="6" t="str">
+        <x:v>mW</x:v>
+      </x:c>
+      <x:c r="D97" s="6" t="str">
+        <x:v>Cota estática con tensión máxima del lado A.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2872,7 +3037,7 @@
         <x:v>SEL-004</x:v>
       </x:c>
       <x:c r="F90" s="6" t="str">
-        <x:v>Tres pull-ups; un pull-down de OE</x:v>
+        <x:v>A1 y B2: 10 kohm a su fuente; OE: 10 kohm a GND; A2Y usa B98.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="60" customHeight="1">
@@ -2892,7 +3057,7 @@
         <x:v>SEL-004</x:v>
       </x:c>
       <x:c r="F91" s="6" t="str">
-        <x:v>1 %; no incluye variación térmica</x:v>
+        <x:v>Tolerancia inicial; coeficiente térmico en B99.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="60" customHeight="1">
@@ -2992,7 +3157,7 @@
         <x:v>SRC-014; §12.1</x:v>
       </x:c>
       <x:c r="F96" s="6" t="str">
-        <x:v>Dos condensadores; referencia exacta por seleccionar</x:v>
+        <x:v>C0603C104K3RACTU: 100 nF, 25 V, X7R; dos unidades.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="60" customHeight="1">
@@ -3013,6 +3178,206 @@
       </x:c>
       <x:c r="F97" s="6" t="str">
         <x:v>Comprobar reducción de potencia con temperatura</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="62" customHeight="1">
+      <x:c r="A98" s="6" t="str">
+        <x:v>Pull-up A2Y / RX Verdin</x:v>
+      </x:c>
+      <x:c r="B98" s="28" t="n">
+        <x:v>47000</x:v>
+      </x:c>
+      <x:c r="C98" s="6" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="D98" s="6" t="str">
+        <x:v>Diseño UART07</x:v>
+      </x:c>
+      <x:c r="E98" s="6" t="str">
+        <x:v>RC0603FR-0747KL</x:v>
+      </x:c>
+      <x:c r="F98" s="6" t="str">
+        <x:v>Sustituye solo el pull-up A2Y de 10 kohm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="62" customHeight="1">
+      <x:c r="A99" s="6" t="str">
+        <x:v>Coeficiente térmico resistencias</x:v>
+      </x:c>
+      <x:c r="B99" s="28" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C99" s="6" t="str">
+        <x:v>ppm/°C</x:v>
+      </x:c>
+      <x:c r="D99" s="6" t="str">
+        <x:v>Ficha YAGEO RC</x:v>
+      </x:c>
+      <x:c r="E99" s="6" t="str">
+        <x:v>RC0603FR-0710KL / 0747KL</x:v>
+      </x:c>
+      <x:c r="F99" s="6" t="str">
+        <x:v>Cota de magnitud</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="62" customHeight="1">
+      <x:c r="A100" s="6" t="str">
+        <x:v>Desviación térmica respecto 25 °C</x:v>
+      </x:c>
+      <x:c r="B100" s="28" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="C100" s="6" t="str">
+        <x:v>°C</x:v>
+      </x:c>
+      <x:c r="D100" s="6" t="str">
+        <x:v>Envolvente -40 a +85 °C</x:v>
+      </x:c>
+      <x:c r="E100" s="6" t="str">
+        <x:v>Diseño UART07</x:v>
+      </x:c>
+      <x:c r="F100" s="6" t="str">
+        <x:v>No incluye envejecimiento</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="62" customHeight="1">
+      <x:c r="A101" s="6" t="str">
+        <x:v>Envolvente A: tensión mínima</x:v>
+      </x:c>
+      <x:c r="B101" s="28" t="n">
+        <x:v>1.65</x:v>
+      </x:c>
+      <x:c r="C101" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D101" s="6" t="str">
+        <x:v>Hipótesis de evaluación</x:v>
+      </x:c>
+      <x:c r="E101" s="6" t="str">
+        <x:v>Diseño UART07</x:v>
+      </x:c>
+      <x:c r="F101" s="6" t="str">
+        <x:v>No es tolerancia garantizada de PWR_1V8_MOCI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="62" customHeight="1">
+      <x:c r="A102" s="6" t="str">
+        <x:v>Fuga conservadora GPIO NXP</x:v>
+      </x:c>
+      <x:c r="B102" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C102" s="6" t="str">
+        <x:v>uA</x:v>
+      </x:c>
+      <x:c r="D102" s="6" t="str">
+        <x:v>NXP IMX8MPIEC rev.2 tabla26</x:v>
+      </x:c>
+      <x:c r="E102" s="6" t="str">
+        <x:v>Fuente en informe</x:v>
+      </x:c>
+      <x:c r="F102" s="6" t="str">
+        <x:v>Deshabilitar pulls internos para el cálculo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="62" customHeight="1">
+      <x:c r="A103" s="6" t="str">
+        <x:v>Fuga TVS a tensión de trabajo</x:v>
+      </x:c>
+      <x:c r="B103" s="28" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="C103" s="6" t="str">
+        <x:v>uA</x:v>
+      </x:c>
+      <x:c r="D103" s="6" t="str">
+        <x:v>TI ESD321 §5.6</x:v>
+      </x:c>
+      <x:c r="E103" s="6" t="str">
+        <x:v>Envolvente térmica de VRWM</x:v>
+      </x:c>
+      <x:c r="F103" s="6" t="str">
+        <x:v>Protección primaria; coordinación pendiente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="62" customHeight="1">
+      <x:c r="A104" s="6" t="str">
+        <x:v>Coeficiente VIH receptor SoC</x:v>
+      </x:c>
+      <x:c r="B104" s="28" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="C104" s="6" t="str">
+        <x:v>V/V</x:v>
+      </x:c>
+      <x:c r="D104" s="6" t="str">
+        <x:v>NXP IMX8MPIEC tabla26</x:v>
+      </x:c>
+      <x:c r="E104" s="6" t="str">
+        <x:v>Fuente en informe</x:v>
+      </x:c>
+      <x:c r="F104" s="6" t="str">
+        <x:v>No aplica a entradas Schmitt del TXU0202</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="62" customHeight="1">
+      <x:c r="A105" s="6" t="str">
+        <x:v>Coeficiente VIL receptor SoC</x:v>
+      </x:c>
+      <x:c r="B105" s="28" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="C105" s="6" t="str">
+        <x:v>V/V</x:v>
+      </x:c>
+      <x:c r="D105" s="6" t="str">
+        <x:v>NXP IMX8MPIEC tabla26</x:v>
+      </x:c>
+      <x:c r="E105" s="6" t="str">
+        <x:v>Fuente en informe</x:v>
+      </x:c>
+      <x:c r="F105" s="6" t="str">
+        <x:v>Carga de salida del traductor ≤100 uA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="62" customHeight="1">
+      <x:c r="A106" s="6" t="str">
+        <x:v>Umbral alto exigido a RX externo</x:v>
+      </x:c>
+      <x:c r="B106" s="28" t="n">
+        <x:v>2.52</x:v>
+      </x:c>
+      <x:c r="C106" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D106" s="6" t="str">
+        <x:v>Contrato externo UART07</x:v>
+      </x:c>
+      <x:c r="E106" s="6" t="str">
+        <x:v>Requisito; no dispositivo ensayado</x:v>
+      </x:c>
+      <x:c r="F106" s="6" t="str">
+        <x:v>Nivel alto reconocido desde este valor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="62" customHeight="1">
+      <x:c r="A107" s="6" t="str">
+        <x:v>Umbral bajo exigido a RX externo</x:v>
+      </x:c>
+      <x:c r="B107" s="28" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="C107" s="6" t="str">
+        <x:v>V</x:v>
+      </x:c>
+      <x:c r="D107" s="6" t="str">
+        <x:v>Contrato externo UART07</x:v>
+      </x:c>
+      <x:c r="E107" s="6" t="str">
+        <x:v>Requisito; no dispositivo ensayado</x:v>
+      </x:c>
+      <x:c r="F107" s="6" t="str">
+        <x:v>Nivel bajo reconocido hasta este valor</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3412,7 +3777,7 @@
         <x:v>Retornos cortos; revisar flancos, carga y referencias de alimentación.</x:v>
       </x:c>
       <x:c r="F19" s="6" t="str">
-        <x:v>Ubicación, GPIO OE y ESD pendientes</x:v>
+        <x:v>OE: X1.206; VCCA: X1.214; coordinación ESD pendiente</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="95" customHeight="1">
@@ -3433,6 +3798,26 @@
       </x:c>
       <x:c r="F20" s="6" t="str">
         <x:v>Requisito externo; no validado físicamente</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="95" customHeight="1">
+      <x:c r="A21" s="6" t="str">
+        <x:v>PCB-16</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="str">
+        <x:v>IF-14/15; SEL-004</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="str">
+        <x:v>Márgenes de entrada TXU0202 sin cierre en toda la envolvente.</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="str">
+        <x:v>Informe UART07; TI §7.5; NXP tabla26</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="str">
+        <x:v>No extrapolar umbrales Schmitt; no certificar inmunidad por rating de TVS.</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="str">
+        <x:v>Captura inicial; liberación bloqueada por revisión eléctrica</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>